<commit_message>
Add calculation of variance for linear case
</commit_message>
<xml_diff>
--- a/Run_array.xlsx
+++ b/Run_array.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jwiegner\ZEN_universe\ZEN-garden-productive\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C69EC0E1-DBD1-44A1-8028-867A10F20A85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49DBF9FA-FE41-420C-9D31-E77E0D911AFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-21720" yWindow="-1965" windowWidth="21840" windowHeight="37920" xr2:uid="{3EBE145F-BAAE-4618-95F6-FEBEE10B4967}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="15">
   <si>
     <t>task_id</t>
   </si>
@@ -493,22 +493,22 @@
         <v>0</v>
       </c>
       <c r="B2" s="1">
-        <v>0</v>
+        <v>2.5000000000000002E-8</v>
       </c>
       <c r="C2" t="b">
         <v>0</v>
       </c>
       <c r="D2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F2" t="s">
         <v>6</v>
       </c>
       <c r="G2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H2" t="s">
         <v>14</v>
@@ -519,7 +519,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="1">
-        <v>2.5000000000000002E-8</v>
+        <v>7.4999999999999997E-8</v>
       </c>
       <c r="C3" t="b">
         <v>0</v>
@@ -545,7 +545,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="1">
-        <v>7.4999999999999997E-8</v>
+        <v>9.9999999999999995E-8</v>
       </c>
       <c r="C4" t="b">
         <v>0</v>
@@ -554,13 +554,13 @@
         <v>1</v>
       </c>
       <c r="E4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F4" t="s">
         <v>6</v>
       </c>
       <c r="G4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H4" t="s">
         <v>14</v>
@@ -574,19 +574,19 @@
         <v>9.9999999999999995E-8</v>
       </c>
       <c r="C5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D5" t="b">
         <v>1</v>
       </c>
       <c r="E5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F5" t="s">
         <v>6</v>
       </c>
       <c r="G5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H5" t="s">
         <v>14</v>
@@ -606,13 +606,13 @@
         <v>1</v>
       </c>
       <c r="E6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F6" t="s">
         <v>6</v>
       </c>
       <c r="G6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="H6" t="s">
         <v>14</v>
@@ -623,7 +623,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="1">
-        <v>9.9999999999999995E-8</v>
+        <v>0</v>
       </c>
       <c r="C7" t="b">
         <v>1</v>
@@ -632,16 +632,13 @@
         <v>1</v>
       </c>
       <c r="E7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F7" t="s">
         <v>6</v>
       </c>
       <c r="G7" t="s">
-        <v>12</v>
-      </c>
-      <c r="H7" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Allow turning parallelization on/off for reevaluation of objective
</commit_message>
<xml_diff>
--- a/Run_array.xlsx
+++ b/Run_array.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jwiegner\ZEN_universe\ZEN-garden-productive\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7C0A391-12F7-41EA-AC56-B0F18358DA9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7909E6C7-A5FC-4E50-92A6-FF27BE6587A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25490" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{3EBE145F-BAAE-4618-95F6-FEBEE10B4967}"/>
+    <workbookView xWindow="1035" yWindow="5430" windowWidth="21810" windowHeight="14055" xr2:uid="{3EBE145F-BAAE-4618-95F6-FEBEE10B4967}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="17">
   <si>
     <t>task_id</t>
   </si>
@@ -62,9 +62,6 @@
     <t>weighting_factor</t>
   </si>
   <si>
-    <t>Comment</t>
-  </si>
-  <si>
     <t>Linear</t>
   </si>
   <si>
@@ -84,6 +81,15 @@
   </si>
   <si>
     <t>x</t>
+  </si>
+  <si>
+    <t>Comment1</t>
+  </si>
+  <si>
+    <t>Comment2</t>
+  </si>
+  <si>
+    <t>Wrong sampling costs</t>
   </si>
 </sst>
 </file>
@@ -456,13 +462,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{86EC76F3-E818-44E9-9042-74C765FA4F6F}">
-  <dimension ref="A1:H17"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:I17"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="13.1796875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="13.140625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -482,13 +488,16 @@
         <v>5</v>
       </c>
       <c r="G1" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="H1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+        <v>12</v>
+      </c>
+      <c r="I1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>0</v>
       </c>
@@ -508,13 +517,16 @@
         <v>6</v>
       </c>
       <c r="G2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="I2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
@@ -534,13 +546,16 @@
         <v>6</v>
       </c>
       <c r="G3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="I3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2</v>
       </c>
@@ -560,13 +575,16 @@
         <v>6</v>
       </c>
       <c r="G4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="I4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>3</v>
       </c>
@@ -586,13 +604,16 @@
         <v>6</v>
       </c>
       <c r="G5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="H5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="I5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>4</v>
       </c>
@@ -612,13 +633,16 @@
         <v>6</v>
       </c>
       <c r="G6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H6" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="I6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>5</v>
       </c>
@@ -638,13 +662,16 @@
         <v>6</v>
       </c>
       <c r="G7" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H7" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="I7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>6</v>
       </c>
@@ -664,13 +691,16 @@
         <v>6</v>
       </c>
       <c r="G8" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H8" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="I8" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>7</v>
       </c>
@@ -690,13 +720,16 @@
         <v>6</v>
       </c>
       <c r="G9" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="I9" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>8</v>
       </c>
@@ -716,13 +749,16 @@
         <v>6</v>
       </c>
       <c r="G10" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H10" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="I10" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>9</v>
       </c>
@@ -742,13 +778,16 @@
         <v>6</v>
       </c>
       <c r="G11" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H11" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="I11" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>10</v>
       </c>
@@ -768,10 +807,16 @@
         <v>6</v>
       </c>
       <c r="G12" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+        <v>8</v>
+      </c>
+      <c r="H12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I12" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>11</v>
       </c>
@@ -791,10 +836,16 @@
         <v>6</v>
       </c>
       <c r="G13" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+        <v>8</v>
+      </c>
+      <c r="H13" t="s">
+        <v>13</v>
+      </c>
+      <c r="I13" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>12</v>
       </c>
@@ -814,10 +865,16 @@
         <v>6</v>
       </c>
       <c r="G14" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+        <v>8</v>
+      </c>
+      <c r="H14" t="s">
+        <v>13</v>
+      </c>
+      <c r="I14" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>13</v>
       </c>
@@ -837,10 +894,16 @@
         <v>6</v>
       </c>
       <c r="G15" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+        <v>8</v>
+      </c>
+      <c r="H15" t="s">
+        <v>13</v>
+      </c>
+      <c r="I15" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>14</v>
       </c>
@@ -860,10 +923,16 @@
         <v>6</v>
       </c>
       <c r="G16" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+        <v>8</v>
+      </c>
+      <c r="H16" t="s">
+        <v>13</v>
+      </c>
+      <c r="I16" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>15</v>
       </c>
@@ -883,7 +952,13 @@
         <v>6</v>
       </c>
       <c r="G17" t="s">
-        <v>9</v>
+        <v>8</v>
+      </c>
+      <c r="H17" t="s">
+        <v>13</v>
+      </c>
+      <c r="I17" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
include correlation for linear case
</commit_message>
<xml_diff>
--- a/Run_array.xlsx
+++ b/Run_array.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jwiegner\ZEN_universe\ZEN-garden-productive\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B267B51-81E0-44A6-99A0-01E5CA75D3B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB68E149-C57F-4A14-840F-8C77B1D58BE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-21720" yWindow="-1965" windowWidth="21840" windowHeight="37920" xr2:uid="{3EBE145F-BAAE-4618-95F6-FEBEE10B4967}"/>
   </bookViews>
@@ -490,7 +490,7 @@
         <v>0</v>
       </c>
       <c r="C2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D2" t="b">
         <v>1</v>

</xml_diff>